<commit_message>
Actualiza chequeo de adjuntos rotos
</commit_message>
<xml_diff>
--- a/reportes/entradas_a_revisar.xlsx
+++ b/reportes/entradas_a_revisar.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
@@ -494,7 +494,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
@@ -525,7 +525,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -556,7 +556,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G5" s="2" t="n"/>
@@ -587,7 +587,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
@@ -618,7 +618,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
@@ -649,7 +649,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -680,7 +680,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G9" s="2" t="n"/>
@@ -711,7 +711,7 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G10" s="2" t="n"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G11" s="2" t="n"/>
@@ -773,7 +773,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G12" s="2" t="n"/>
@@ -804,7 +804,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G13" s="2" t="n"/>
@@ -835,7 +835,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G14" s="2" t="n"/>
@@ -866,7 +866,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G15" s="2" t="n"/>
@@ -897,7 +897,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G16" s="2" t="n"/>
@@ -928,7 +928,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G17" s="2" t="n"/>
@@ -959,7 +959,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
@@ -990,7 +990,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G19" s="2" t="n"/>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G20" s="2" t="n"/>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G21" s="2" t="n"/>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G22" s="2" t="n"/>
@@ -1116,7 +1116,7 @@
       <c r="E23" s="4" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G23" s="2" t="n"/>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G24" s="2" t="n"/>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G25" s="2" t="n"/>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G26" s="2" t="n"/>
@@ -1242,7 +1242,7 @@
       <c r="E27" s="4" t="inlineStr"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G27" s="2" t="n"/>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G28" s="2" t="n"/>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G29" s="2" t="n"/>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G30" s="2" t="n"/>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G31" s="2" t="n"/>
@@ -1397,7 +1397,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G32" s="2" t="n"/>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G33" s="2" t="n"/>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G34" s="2" t="n"/>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G35" s="2" t="n"/>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G36" s="2" t="n"/>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G37" s="2" t="n"/>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G38" s="2" t="n"/>
@@ -1616,7 +1616,7 @@
       <c r="E39" s="4" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G39" s="2" t="n"/>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G40" s="2" t="n"/>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G41" s="2" t="n"/>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G42" s="2" t="n"/>
@@ -1742,7 +1742,7 @@
       <c r="E43" s="4" t="inlineStr"/>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G43" s="2" t="n"/>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G44" s="2" t="n"/>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G45" s="2" t="n"/>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G46" s="2" t="n"/>
@@ -1866,7 +1866,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G47" s="2" t="n"/>
@@ -1899,7 +1899,7 @@
       <c r="E48" s="4" t="inlineStr"/>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G48" s="2" t="n"/>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G49" s="2" t="n"/>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G50" s="2" t="n"/>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G51" s="2" t="n"/>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G52" s="2" t="n"/>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G53" s="2" t="n"/>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G54" s="2" t="n"/>
@@ -2118,7 +2118,7 @@
       <c r="E55" s="4" t="inlineStr"/>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G55" s="2" t="n"/>
@@ -2151,7 +2151,7 @@
       <c r="E56" s="4" t="inlineStr"/>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G56" s="2" t="n"/>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G57" s="2" t="n"/>
@@ -2213,7 +2213,7 @@
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G58" s="2" t="n"/>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G59" s="2" t="n"/>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G60" s="2" t="n"/>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G61" s="2" t="n"/>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G62" s="2" t="n"/>
@@ -2368,7 +2368,7 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G63" s="2" t="n"/>
@@ -2399,7 +2399,7 @@
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G64" s="2" t="n"/>
@@ -2430,7 +2430,7 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G65" s="2" t="n"/>
@@ -2463,7 +2463,7 @@
       <c r="E66" s="4" t="inlineStr"/>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G66" s="2" t="n"/>
@@ -2494,7 +2494,7 @@
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G67" s="2" t="n"/>
@@ -2525,7 +2525,7 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G68" s="2" t="n"/>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G69" s="2" t="n"/>
@@ -2589,7 +2589,7 @@
       <c r="E70" s="4" t="inlineStr"/>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G70" s="2" t="n"/>
@@ -2622,7 +2622,7 @@
       <c r="E71" s="4" t="inlineStr"/>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G71" s="2" t="n"/>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G72" s="2" t="n"/>
@@ -2684,7 +2684,7 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G73" s="2" t="n"/>
@@ -2715,7 +2715,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G74" s="2" t="n"/>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G75" s="2" t="n"/>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G76" s="2" t="n"/>
@@ -2808,7 +2808,7 @@
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G77" s="2" t="n"/>
@@ -2841,7 +2841,7 @@
       <c r="E78" s="4" t="inlineStr"/>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G78" s="2" t="n"/>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G79" s="2" t="n"/>
@@ -2905,7 +2905,7 @@
       <c r="E80" s="4" t="inlineStr"/>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G80" s="2" t="n"/>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G81" s="2" t="n"/>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G82" s="2" t="n"/>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G83" s="2" t="n"/>
@@ -3031,7 +3031,7 @@
       <c r="E84" s="4" t="inlineStr"/>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G84" s="2" t="n"/>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G85" s="2" t="n"/>
@@ -3095,7 +3095,7 @@
       <c r="E86" s="4" t="inlineStr"/>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G86" s="2" t="n"/>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G87" s="2" t="n"/>
@@ -3157,7 +3157,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G88" s="2" t="n"/>
@@ -3190,7 +3190,7 @@
       <c r="E89" s="4" t="inlineStr"/>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G89" s="2" t="n"/>
@@ -3221,7 +3221,7 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G90" s="2" t="n"/>
@@ -3252,7 +3252,7 @@
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G91" s="2" t="n"/>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="F92" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G92" s="2" t="n"/>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G93" s="2" t="n"/>
@@ -3345,7 +3345,7 @@
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G94" s="2" t="n"/>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G95" s="2" t="n"/>
@@ -3409,7 +3409,7 @@
       <c r="E96" s="4" t="inlineStr"/>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G96" s="2" t="n"/>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G97" s="2" t="n"/>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G98" s="2" t="n"/>
@@ -3504,7 +3504,7 @@
       <c r="E99" s="4" t="inlineStr"/>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G99" s="2" t="n"/>
@@ -3535,7 +3535,7 @@
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G100" s="2" t="n"/>
@@ -3568,7 +3568,7 @@
       <c r="E101" s="4" t="inlineStr"/>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G101" s="2" t="n"/>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G102" s="2" t="n"/>
@@ -3630,7 +3630,7 @@
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G103" s="2" t="n"/>
@@ -3663,7 +3663,7 @@
       <c r="E104" s="4" t="inlineStr"/>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G104" s="2" t="n"/>
@@ -3696,7 +3696,7 @@
       <c r="E105" s="4" t="inlineStr"/>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G105" s="2" t="n"/>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G106" s="2" t="n"/>
@@ -3758,7 +3758,7 @@
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G107" s="2" t="n"/>
@@ -3789,7 +3789,7 @@
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G108" s="2" t="n"/>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G109" s="2" t="n"/>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="F110" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G110" s="2" t="n"/>
@@ -3882,7 +3882,7 @@
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G111" s="2" t="n"/>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G112" s="2" t="n"/>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G113" s="2" t="n"/>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G114" s="2" t="n"/>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G115" s="2" t="n"/>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G116" s="2" t="n"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G117" s="2" t="n"/>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="F118" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G118" s="2" t="n"/>
@@ -4132,7 +4132,7 @@
       <c r="E119" s="4" t="inlineStr"/>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G119" s="2" t="n"/>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="F120" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G120" s="2" t="n"/>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G121" s="2" t="n"/>
@@ -4225,7 +4225,7 @@
       </c>
       <c r="F122" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G122" s="2" t="n"/>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G123" s="2" t="n"/>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G124" s="2" t="n"/>
@@ -4320,7 +4320,7 @@
       <c r="E125" s="4" t="inlineStr"/>
       <c r="F125" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G125" s="2" t="n"/>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G126" s="2" t="n"/>
@@ -4382,7 +4382,7 @@
       </c>
       <c r="F127" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G127" s="2" t="n"/>
@@ -4415,7 +4415,7 @@
       <c r="E128" s="4" t="inlineStr"/>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G128" s="2" t="n"/>
@@ -4448,7 +4448,7 @@
       <c r="E129" s="4" t="inlineStr"/>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G129" s="2" t="n"/>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G130" s="2" t="n"/>
@@ -4512,7 +4512,7 @@
       <c r="E131" s="4" t="inlineStr"/>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G131" s="2" t="n"/>
@@ -4543,7 +4543,7 @@
       </c>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G132" s="2" t="n"/>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G133" s="2" t="n"/>
@@ -4605,7 +4605,7 @@
       </c>
       <c r="F134" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G134" s="2" t="n"/>
@@ -4636,7 +4636,7 @@
       </c>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G135" s="2" t="n"/>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="F136" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G136" s="2" t="n"/>
@@ -4698,7 +4698,7 @@
       </c>
       <c r="F137" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G137" s="2" t="n"/>
@@ -4729,7 +4729,7 @@
       </c>
       <c r="F138" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G138" s="2" t="n"/>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G139" s="2" t="n"/>
@@ -4793,7 +4793,7 @@
       <c r="E140" s="4" t="inlineStr"/>
       <c r="F140" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G140" s="2" t="n"/>
@@ -4824,7 +4824,7 @@
       </c>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G141" s="2" t="n"/>
@@ -4855,7 +4855,7 @@
       </c>
       <c r="F142" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G142" s="2" t="n"/>
@@ -4886,7 +4886,7 @@
       </c>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G143" s="2" t="n"/>
@@ -4917,7 +4917,7 @@
       </c>
       <c r="F144" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G144" s="2" t="n"/>
@@ -4950,7 +4950,7 @@
       <c r="E145" s="4" t="inlineStr"/>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G145" s="2" t="n"/>
@@ -4981,7 +4981,7 @@
       </c>
       <c r="F146" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G146" s="2" t="n"/>
@@ -5012,7 +5012,7 @@
       </c>
       <c r="F147" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G147" s="2" t="n"/>
@@ -5045,7 +5045,7 @@
       <c r="E148" s="4" t="inlineStr"/>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G148" s="2" t="n"/>
@@ -5078,7 +5078,7 @@
       <c r="E149" s="4" t="inlineStr"/>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G149" s="2" t="n"/>
@@ -5111,7 +5111,7 @@
       <c r="E150" s="4" t="inlineStr"/>
       <c r="F150" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G150" s="2" t="n"/>
@@ -5144,7 +5144,7 @@
       <c r="E151" s="4" t="inlineStr"/>
       <c r="F151" s="3" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G151" s="2" t="n"/>
@@ -5175,7 +5175,7 @@
       </c>
       <c r="F152" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G152" s="2" t="n"/>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="F153" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G153" s="2" t="n"/>
@@ -5237,7 +5237,7 @@
       </c>
       <c r="F154" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G154" s="2" t="n"/>
@@ -5268,7 +5268,7 @@
       </c>
       <c r="F155" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G155" s="2" t="n"/>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="F156" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G156" s="2" t="n"/>
@@ -5330,7 +5330,7 @@
       </c>
       <c r="F157" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G157" s="2" t="n"/>
@@ -5361,7 +5361,7 @@
       </c>
       <c r="F158" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G158" s="2" t="n"/>
@@ -5392,7 +5392,7 @@
       </c>
       <c r="F159" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G159" s="2" t="n"/>
@@ -5423,7 +5423,7 @@
       </c>
       <c r="F160" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G160" s="2" t="n"/>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="F161" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G161" s="2" t="n"/>
@@ -5485,7 +5485,7 @@
       </c>
       <c r="F162" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G162" s="2" t="n"/>
@@ -5516,7 +5516,7 @@
       </c>
       <c r="F163" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G163" s="2" t="n"/>
@@ -5547,7 +5547,7 @@
       </c>
       <c r="F164" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G164" s="2" t="n"/>
@@ -5578,7 +5578,7 @@
       </c>
       <c r="F165" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G165" s="2" t="n"/>
@@ -5609,7 +5609,7 @@
       </c>
       <c r="F166" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G166" s="2" t="n"/>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="F167" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G167" s="2" t="n"/>
@@ -5671,7 +5671,7 @@
       </c>
       <c r="F168" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G168" s="2" t="n"/>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="F169" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G169" s="2" t="n"/>
@@ -5733,7 +5733,7 @@
       </c>
       <c r="F170" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G170" s="2" t="n"/>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="F171" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G171" s="2" t="n"/>
@@ -5795,7 +5795,7 @@
       </c>
       <c r="F172" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G172" s="2" t="n"/>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="F173" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G173" s="2" t="n"/>
@@ -5857,7 +5857,7 @@
       </c>
       <c r="F174" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G174" s="2" t="n"/>
@@ -5888,7 +5888,7 @@
       </c>
       <c r="F175" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G175" s="2" t="n"/>
@@ -5919,7 +5919,7 @@
       </c>
       <c r="F176" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G176" s="2" t="n"/>
@@ -5950,7 +5950,7 @@
       </c>
       <c r="F177" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G177" s="2" t="n"/>
@@ -5981,7 +5981,7 @@
       </c>
       <c r="F178" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G178" s="2" t="n"/>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="F179" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G179" s="2" t="n"/>
@@ -6043,7 +6043,7 @@
       </c>
       <c r="F180" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G180" s="2" t="n"/>
@@ -6074,7 +6074,7 @@
       </c>
       <c r="F181" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G181" s="2" t="n"/>
@@ -6105,7 +6105,7 @@
       </c>
       <c r="F182" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G182" s="2" t="n"/>
@@ -6136,7 +6136,7 @@
       </c>
       <c r="F183" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G183" s="2" t="n"/>
@@ -6167,7 +6167,7 @@
       </c>
       <c r="F184" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G184" s="2" t="n"/>
@@ -6198,7 +6198,7 @@
       </c>
       <c r="F185" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G185" s="2" t="n"/>
@@ -6229,7 +6229,7 @@
       </c>
       <c r="F186" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G186" s="2" t="n"/>
@@ -6260,7 +6260,7 @@
       </c>
       <c r="F187" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G187" s="2" t="n"/>
@@ -6291,7 +6291,7 @@
       </c>
       <c r="F188" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G188" s="2" t="n"/>
@@ -6322,7 +6322,7 @@
       </c>
       <c r="F189" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G189" s="2" t="n"/>
@@ -6353,7 +6353,7 @@
       </c>
       <c r="F190" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G190" s="2" t="n"/>
@@ -6384,7 +6384,7 @@
       </c>
       <c r="F191" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G191" s="2" t="n"/>
@@ -6415,7 +6415,7 @@
       </c>
       <c r="F192" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G192" s="2" t="n"/>
@@ -6446,7 +6446,7 @@
       </c>
       <c r="F193" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G193" s="2" t="n"/>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="F194" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G194" s="2" t="n"/>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="F195" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G195" s="2" t="n"/>
@@ -6539,7 +6539,7 @@
       </c>
       <c r="F196" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G196" s="2" t="n"/>
@@ -6570,7 +6570,7 @@
       </c>
       <c r="F197" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G197" s="2" t="n"/>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="F198" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G198" s="2" t="n"/>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="F199" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G199" s="2" t="n"/>
@@ -6663,7 +6663,7 @@
       </c>
       <c r="F200" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G200" s="2" t="n"/>
@@ -6694,7 +6694,7 @@
       </c>
       <c r="F201" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G201" s="2" t="n"/>
@@ -6725,7 +6725,7 @@
       </c>
       <c r="F202" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G202" s="2" t="n"/>
@@ -6756,7 +6756,7 @@
       </c>
       <c r="F203" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G203" s="2" t="n"/>
@@ -6787,7 +6787,7 @@
       </c>
       <c r="F204" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G204" s="2" t="n"/>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="F205" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G205" s="2" t="n"/>
@@ -6849,7 +6849,7 @@
       </c>
       <c r="F206" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G206" s="2" t="n"/>
@@ -6880,7 +6880,7 @@
       </c>
       <c r="F207" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G207" s="2" t="n"/>
@@ -6911,7 +6911,7 @@
       </c>
       <c r="F208" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G208" s="2" t="n"/>
@@ -6942,7 +6942,7 @@
       </c>
       <c r="F209" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G209" s="2" t="n"/>
@@ -6973,7 +6973,7 @@
       </c>
       <c r="F210" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G210" s="2" t="n"/>
@@ -7004,7 +7004,7 @@
       </c>
       <c r="F211" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G211" s="2" t="n"/>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="F212" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G212" s="2" t="n"/>
@@ -7066,7 +7066,7 @@
       </c>
       <c r="F213" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G213" s="2" t="n"/>
@@ -7097,7 +7097,7 @@
       </c>
       <c r="F214" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G214" s="2" t="n"/>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="F215" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G215" s="2" t="n"/>
@@ -7159,7 +7159,7 @@
       </c>
       <c r="F216" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G216" s="2" t="n"/>
@@ -7190,7 +7190,7 @@
       </c>
       <c r="F217" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G217" s="2" t="n"/>
@@ -7221,7 +7221,7 @@
       </c>
       <c r="F218" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G218" s="2" t="n"/>
@@ -7252,7 +7252,7 @@
       </c>
       <c r="F219" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G219" s="2" t="n"/>
@@ -7283,7 +7283,7 @@
       </c>
       <c r="F220" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G220" s="2" t="n"/>
@@ -7314,7 +7314,7 @@
       </c>
       <c r="F221" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G221" s="2" t="n"/>
@@ -7345,7 +7345,7 @@
       </c>
       <c r="F222" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G222" s="2" t="n"/>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="F223" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G223" s="2" t="n"/>
@@ -7407,7 +7407,7 @@
       </c>
       <c r="F224" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G224" s="2" t="n"/>
@@ -7438,7 +7438,7 @@
       </c>
       <c r="F225" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G225" s="2" t="n"/>
@@ -7469,7 +7469,7 @@
       </c>
       <c r="F226" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G226" s="2" t="n"/>
@@ -7500,7 +7500,7 @@
       </c>
       <c r="F227" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G227" s="2" t="n"/>
@@ -7531,7 +7531,7 @@
       </c>
       <c r="F228" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G228" s="2" t="n"/>
@@ -7562,7 +7562,7 @@
       </c>
       <c r="F229" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G229" s="2" t="n"/>
@@ -7593,7 +7593,7 @@
       </c>
       <c r="F230" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G230" s="2" t="n"/>
@@ -7624,7 +7624,7 @@
       </c>
       <c r="F231" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G231" s="2" t="n"/>
@@ -7655,7 +7655,7 @@
       </c>
       <c r="F232" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G232" s="2" t="n"/>
@@ -7686,7 +7686,7 @@
       </c>
       <c r="F233" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G233" s="2" t="n"/>
@@ -7717,7 +7717,7 @@
       </c>
       <c r="F234" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G234" s="2" t="n"/>
@@ -7748,7 +7748,7 @@
       </c>
       <c r="F235" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G235" s="2" t="n"/>
@@ -7779,7 +7779,7 @@
       </c>
       <c r="F236" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G236" s="2" t="n"/>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="F237" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G237" s="2" t="n"/>
@@ -7841,7 +7841,7 @@
       </c>
       <c r="F238" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G238" s="2" t="n"/>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="F239" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G239" s="2" t="n"/>
@@ -7903,7 +7903,7 @@
       </c>
       <c r="F240" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G240" s="2" t="n"/>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="F241" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G241" s="2" t="n"/>
@@ -7965,7 +7965,7 @@
       </c>
       <c r="F242" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G242" s="2" t="n"/>
@@ -7996,7 +7996,7 @@
       </c>
       <c r="F243" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G243" s="2" t="n"/>
@@ -8027,7 +8027,7 @@
       </c>
       <c r="F244" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G244" s="2" t="n"/>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="F245" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G245" s="2" t="n"/>
@@ -8089,7 +8089,7 @@
       </c>
       <c r="F246" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G246" s="2" t="n"/>
@@ -8120,7 +8120,7 @@
       </c>
       <c r="F247" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G247" s="2" t="n"/>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="F248" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G248" s="2" t="n"/>
@@ -8182,7 +8182,7 @@
       </c>
       <c r="F249" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G249" s="2" t="n"/>
@@ -8213,7 +8213,7 @@
       </c>
       <c r="F250" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G250" s="2" t="n"/>
@@ -8246,7 +8246,7 @@
       <c r="E251" s="6" t="inlineStr"/>
       <c r="F251" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G251" s="2" t="n"/>
@@ -8277,7 +8277,7 @@
       </c>
       <c r="F252" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G252" s="2" t="n"/>
@@ -8308,7 +8308,7 @@
       </c>
       <c r="F253" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G253" s="2" t="n"/>
@@ -8339,7 +8339,7 @@
       </c>
       <c r="F254" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G254" s="2" t="n"/>
@@ -8370,7 +8370,7 @@
       </c>
       <c r="F255" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G255" s="2" t="n"/>
@@ -8401,7 +8401,7 @@
       </c>
       <c r="F256" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G256" s="2" t="n"/>
@@ -8432,7 +8432,7 @@
       </c>
       <c r="F257" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G257" s="2" t="n"/>
@@ -8463,7 +8463,7 @@
       </c>
       <c r="F258" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G258" s="2" t="n"/>
@@ -8494,7 +8494,7 @@
       </c>
       <c r="F259" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G259" s="2" t="n"/>
@@ -8525,7 +8525,7 @@
       </c>
       <c r="F260" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G260" s="2" t="n"/>
@@ -8556,7 +8556,7 @@
       </c>
       <c r="F261" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G261" s="2" t="n"/>
@@ -8587,7 +8587,7 @@
       </c>
       <c r="F262" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G262" s="2" t="n"/>
@@ -8618,7 +8618,7 @@
       </c>
       <c r="F263" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G263" s="2" t="n"/>
@@ -8649,7 +8649,7 @@
       </c>
       <c r="F264" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G264" s="2" t="n"/>
@@ -8680,7 +8680,7 @@
       </c>
       <c r="F265" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G265" s="2" t="n"/>
@@ -8711,7 +8711,7 @@
       </c>
       <c r="F266" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G266" s="2" t="n"/>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="F267" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G267" s="2" t="n"/>
@@ -8773,7 +8773,7 @@
       </c>
       <c r="F268" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G268" s="2" t="n"/>
@@ -8804,7 +8804,7 @@
       </c>
       <c r="F269" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G269" s="2" t="n"/>
@@ -8835,7 +8835,7 @@
       </c>
       <c r="F270" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G270" s="2" t="n"/>
@@ -8866,7 +8866,7 @@
       </c>
       <c r="F271" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G271" s="2" t="n"/>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="F272" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G272" s="2" t="n"/>
@@ -8928,7 +8928,7 @@
       </c>
       <c r="F273" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G273" s="2" t="n"/>
@@ -8959,7 +8959,7 @@
       </c>
       <c r="F274" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G274" s="2" t="n"/>
@@ -8990,7 +8990,7 @@
       </c>
       <c r="F275" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G275" s="2" t="n"/>
@@ -9021,7 +9021,7 @@
       </c>
       <c r="F276" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G276" s="2" t="n"/>
@@ -9052,7 +9052,7 @@
       </c>
       <c r="F277" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G277" s="2" t="n"/>
@@ -9083,7 +9083,7 @@
       </c>
       <c r="F278" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G278" s="2" t="n"/>
@@ -9114,7 +9114,7 @@
       </c>
       <c r="F279" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G279" s="2" t="n"/>
@@ -9145,7 +9145,7 @@
       </c>
       <c r="F280" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G280" s="2" t="n"/>
@@ -9176,7 +9176,7 @@
       </c>
       <c r="F281" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G281" s="2" t="n"/>
@@ -9207,7 +9207,7 @@
       </c>
       <c r="F282" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G282" s="2" t="n"/>
@@ -9238,7 +9238,7 @@
       </c>
       <c r="F283" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G283" s="2" t="n"/>
@@ -9269,7 +9269,7 @@
       </c>
       <c r="F284" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G284" s="2" t="n"/>
@@ -9300,7 +9300,7 @@
       </c>
       <c r="F285" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G285" s="2" t="n"/>
@@ -9331,7 +9331,7 @@
       </c>
       <c r="F286" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G286" s="2" t="n"/>
@@ -9362,7 +9362,7 @@
       </c>
       <c r="F287" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G287" s="2" t="n"/>
@@ -9393,7 +9393,7 @@
       </c>
       <c r="F288" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G288" s="2" t="n"/>
@@ -9424,7 +9424,7 @@
       </c>
       <c r="F289" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G289" s="2" t="n"/>
@@ -9455,7 +9455,7 @@
       </c>
       <c r="F290" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G290" s="2" t="n"/>
@@ -9486,7 +9486,7 @@
       </c>
       <c r="F291" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G291" s="2" t="n"/>
@@ -9517,7 +9517,7 @@
       </c>
       <c r="F292" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G292" s="2" t="n"/>
@@ -9548,7 +9548,7 @@
       </c>
       <c r="F293" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G293" s="2" t="n"/>
@@ -9579,7 +9579,7 @@
       </c>
       <c r="F294" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G294" s="2" t="n"/>
@@ -9610,7 +9610,7 @@
       </c>
       <c r="F295" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G295" s="2" t="n"/>
@@ -9641,7 +9641,7 @@
       </c>
       <c r="F296" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G296" s="2" t="n"/>
@@ -9672,7 +9672,7 @@
       </c>
       <c r="F297" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G297" s="2" t="n"/>
@@ -9703,7 +9703,7 @@
       </c>
       <c r="F298" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G298" s="2" t="n"/>
@@ -9734,7 +9734,7 @@
       </c>
       <c r="F299" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G299" s="2" t="n"/>
@@ -9765,7 +9765,7 @@
       </c>
       <c r="F300" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G300" s="2" t="n"/>
@@ -9796,7 +9796,7 @@
       </c>
       <c r="F301" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G301" s="2" t="n"/>
@@ -9827,7 +9827,7 @@
       </c>
       <c r="F302" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G302" s="2" t="n"/>
@@ -9858,7 +9858,7 @@
       </c>
       <c r="F303" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G303" s="2" t="n"/>
@@ -9889,7 +9889,7 @@
       </c>
       <c r="F304" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G304" s="2" t="n"/>
@@ -9920,7 +9920,7 @@
       </c>
       <c r="F305" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G305" s="2" t="n"/>
@@ -9951,7 +9951,7 @@
       </c>
       <c r="F306" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G306" s="2" t="n"/>
@@ -9982,7 +9982,7 @@
       </c>
       <c r="F307" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G307" s="2" t="n"/>
@@ -10013,7 +10013,7 @@
       </c>
       <c r="F308" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G308" s="2" t="n"/>
@@ -10044,7 +10044,7 @@
       </c>
       <c r="F309" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G309" s="2" t="n"/>
@@ -10075,7 +10075,7 @@
       </c>
       <c r="F310" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G310" s="2" t="n"/>
@@ -10106,7 +10106,7 @@
       </c>
       <c r="F311" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G311" s="2" t="n"/>
@@ -10137,7 +10137,7 @@
       </c>
       <c r="F312" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G312" s="2" t="n"/>
@@ -10168,7 +10168,7 @@
       </c>
       <c r="F313" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G313" s="2" t="n"/>
@@ -10199,7 +10199,7 @@
       </c>
       <c r="F314" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G314" s="2" t="n"/>
@@ -10230,7 +10230,7 @@
       </c>
       <c r="F315" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G315" s="2" t="n"/>
@@ -10261,7 +10261,7 @@
       </c>
       <c r="F316" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G316" s="2" t="n"/>
@@ -10292,7 +10292,7 @@
       </c>
       <c r="F317" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G317" s="2" t="n"/>
@@ -10323,7 +10323,7 @@
       </c>
       <c r="F318" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G318" s="2" t="n"/>
@@ -10354,7 +10354,7 @@
       </c>
       <c r="F319" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G319" s="2" t="n"/>
@@ -10385,7 +10385,7 @@
       </c>
       <c r="F320" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G320" s="2" t="n"/>
@@ -10416,7 +10416,7 @@
       </c>
       <c r="F321" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G321" s="2" t="n"/>
@@ -10447,7 +10447,7 @@
       </c>
       <c r="F322" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G322" s="2" t="n"/>
@@ -10478,7 +10478,7 @@
       </c>
       <c r="F323" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G323" s="2" t="n"/>
@@ -10509,7 +10509,7 @@
       </c>
       <c r="F324" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G324" s="2" t="n"/>
@@ -10540,7 +10540,7 @@
       </c>
       <c r="F325" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G325" s="2" t="n"/>
@@ -10571,7 +10571,7 @@
       </c>
       <c r="F326" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G326" s="2" t="n"/>
@@ -10602,7 +10602,7 @@
       </c>
       <c r="F327" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G327" s="2" t="n"/>
@@ -10633,7 +10633,7 @@
       </c>
       <c r="F328" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G328" s="2" t="n"/>
@@ -10664,7 +10664,7 @@
       </c>
       <c r="F329" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G329" s="2" t="n"/>
@@ -10695,7 +10695,7 @@
       </c>
       <c r="F330" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G330" s="2" t="n"/>
@@ -10726,7 +10726,7 @@
       </c>
       <c r="F331" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G331" s="2" t="n"/>
@@ -10757,7 +10757,7 @@
       </c>
       <c r="F332" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G332" s="2" t="n"/>
@@ -10788,7 +10788,7 @@
       </c>
       <c r="F333" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G333" s="2" t="n"/>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="F334" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G334" s="2" t="n"/>
@@ -10850,7 +10850,7 @@
       </c>
       <c r="F335" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G335" s="2" t="n"/>
@@ -10881,7 +10881,7 @@
       </c>
       <c r="F336" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G336" s="2" t="n"/>
@@ -10912,7 +10912,7 @@
       </c>
       <c r="F337" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G337" s="2" t="n"/>
@@ -10943,7 +10943,7 @@
       </c>
       <c r="F338" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G338" s="2" t="n"/>
@@ -10974,7 +10974,7 @@
       </c>
       <c r="F339" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G339" s="2" t="n"/>
@@ -11005,7 +11005,7 @@
       </c>
       <c r="F340" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G340" s="2" t="n"/>
@@ -11036,7 +11036,7 @@
       </c>
       <c r="F341" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G341" s="2" t="n"/>
@@ -11067,7 +11067,7 @@
       </c>
       <c r="F342" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G342" s="2" t="n"/>
@@ -11098,7 +11098,7 @@
       </c>
       <c r="F343" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G343" s="2" t="n"/>
@@ -11129,7 +11129,7 @@
       </c>
       <c r="F344" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G344" s="2" t="n"/>
@@ -11160,7 +11160,7 @@
       </c>
       <c r="F345" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G345" s="2" t="n"/>
@@ -11191,7 +11191,7 @@
       </c>
       <c r="F346" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G346" s="2" t="n"/>
@@ -11222,7 +11222,7 @@
       </c>
       <c r="F347" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G347" s="2" t="n"/>
@@ -11253,7 +11253,7 @@
       </c>
       <c r="F348" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G348" s="2" t="n"/>
@@ -11284,7 +11284,7 @@
       </c>
       <c r="F349" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G349" s="2" t="n"/>
@@ -11315,7 +11315,7 @@
       </c>
       <c r="F350" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G350" s="2" t="n"/>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="F351" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G351" s="2" t="n"/>
@@ -11377,7 +11377,7 @@
       </c>
       <c r="F352" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G352" s="2" t="n"/>
@@ -11408,7 +11408,7 @@
       </c>
       <c r="F353" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G353" s="2" t="n"/>
@@ -11439,7 +11439,7 @@
       </c>
       <c r="F354" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G354" s="2" t="n"/>
@@ -11470,7 +11470,7 @@
       </c>
       <c r="F355" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G355" s="2" t="n"/>
@@ -11501,7 +11501,7 @@
       </c>
       <c r="F356" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G356" s="2" t="n"/>
@@ -11532,7 +11532,7 @@
       </c>
       <c r="F357" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G357" s="2" t="n"/>
@@ -11567,7 +11567,7 @@
       </c>
       <c r="F358" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G358" s="2" t="n"/>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="F359" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G359" s="2" t="n"/>
@@ -11629,7 +11629,7 @@
       </c>
       <c r="F360" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G360" s="2" t="n"/>
@@ -11660,7 +11660,7 @@
       </c>
       <c r="F361" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G361" s="2" t="n"/>
@@ -11691,7 +11691,7 @@
       </c>
       <c r="F362" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G362" s="2" t="n"/>
@@ -11722,7 +11722,7 @@
       </c>
       <c r="F363" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G363" s="2" t="n"/>
@@ -11753,7 +11753,7 @@
       </c>
       <c r="F364" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G364" s="2" t="n"/>
@@ -11784,7 +11784,7 @@
       </c>
       <c r="F365" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G365" s="2" t="n"/>
@@ -11815,7 +11815,7 @@
       </c>
       <c r="F366" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G366" s="2" t="n"/>
@@ -11846,7 +11846,7 @@
       </c>
       <c r="F367" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G367" s="2" t="n"/>
@@ -11877,7 +11877,7 @@
       </c>
       <c r="F368" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G368" s="2" t="n"/>
@@ -11908,7 +11908,7 @@
       </c>
       <c r="F369" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G369" s="2" t="n"/>
@@ -11939,7 +11939,7 @@
       </c>
       <c r="F370" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G370" s="2" t="n"/>
@@ -11970,7 +11970,7 @@
       </c>
       <c r="F371" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G371" s="2" t="n"/>
@@ -12001,7 +12001,7 @@
       </c>
       <c r="F372" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G372" s="2" t="n"/>
@@ -12032,7 +12032,7 @@
       </c>
       <c r="F373" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G373" s="2" t="n"/>
@@ -12063,7 +12063,7 @@
       </c>
       <c r="F374" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G374" s="2" t="n"/>
@@ -12094,7 +12094,7 @@
       </c>
       <c r="F375" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G375" s="2" t="n"/>
@@ -12125,7 +12125,7 @@
       </c>
       <c r="F376" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G376" s="2" t="n"/>
@@ -12156,7 +12156,7 @@
       </c>
       <c r="F377" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G377" s="2" t="n"/>
@@ -12187,7 +12187,7 @@
       </c>
       <c r="F378" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G378" s="2" t="n"/>
@@ -12218,7 +12218,7 @@
       </c>
       <c r="F379" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G379" s="2" t="n"/>
@@ -12249,7 +12249,7 @@
       </c>
       <c r="F380" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G380" s="2" t="n"/>
@@ -12280,7 +12280,7 @@
       </c>
       <c r="F381" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G381" s="2" t="n"/>
@@ -12311,7 +12311,7 @@
       </c>
       <c r="F382" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G382" s="2" t="n"/>
@@ -12342,7 +12342,7 @@
       </c>
       <c r="F383" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G383" s="2" t="n"/>
@@ -12373,7 +12373,7 @@
       </c>
       <c r="F384" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G384" s="2" t="n"/>
@@ -12404,7 +12404,7 @@
       </c>
       <c r="F385" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G385" s="2" t="n"/>
@@ -12435,7 +12435,7 @@
       </c>
       <c r="F386" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G386" s="2" t="n"/>
@@ -12466,7 +12466,7 @@
       </c>
       <c r="F387" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G387" s="2" t="n"/>
@@ -12497,7 +12497,7 @@
       </c>
       <c r="F388" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G388" s="2" t="n"/>
@@ -12528,7 +12528,7 @@
       </c>
       <c r="F389" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G389" s="2" t="n"/>
@@ -12559,7 +12559,7 @@
       </c>
       <c r="F390" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G390" s="2" t="n"/>
@@ -12590,7 +12590,7 @@
       </c>
       <c r="F391" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G391" s="2" t="n"/>
@@ -12621,7 +12621,7 @@
       </c>
       <c r="F392" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G392" s="2" t="n"/>
@@ -12652,7 +12652,7 @@
       </c>
       <c r="F393" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G393" s="2" t="n"/>
@@ -12683,7 +12683,7 @@
       </c>
       <c r="F394" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G394" s="2" t="n"/>
@@ -12714,7 +12714,7 @@
       </c>
       <c r="F395" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G395" s="2" t="n"/>
@@ -12745,7 +12745,7 @@
       </c>
       <c r="F396" s="6" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="G396" s="2" t="n"/>

</xml_diff>